<commit_message>
feat(upload): expand master Excel schemas with full operational columns
Product master now requires group, type, short/full name, UoM, and main storage location; other masters enriched with optional fields and legacy header aliases.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/qa/upload-templates/bom_upload_template.xlsx
+++ b/docs/qa/upload-templates/bom_upload_template.xlsx
@@ -133,7 +133,7 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Parent FG code (must exist in Product Master)</t>
+        <t>Parent FG/SFG code (must exist in Product Master)</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
@@ -144,6 +144,11 @@
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
         <t>Numeric &gt;= 0</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>Component UoM</t>
       </text>
     </comment>
   </commentList>
@@ -439,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -460,7 +465,27 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>uom</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>scrap_pct</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>operation_seq</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>effective_from</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>effective_to</t>
         </is>
       </c>
     </row>
@@ -478,9 +503,23 @@
       <c r="C2" t="n">
         <v>8.5</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
         <v>2</v>
       </c>
+      <c r="F2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -490,15 +529,29 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>RM-CORE</t>
+          <t>SF-CORE100</t>
         </is>
       </c>
       <c r="C3" t="n">
         <v>1</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
         <v>0</v>
       </c>
+      <c r="F3" t="n">
+        <v>20</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -514,9 +567,23 @@
       <c r="C4" t="n">
         <v>14</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
         <v>2</v>
       </c>
+      <c r="F4" t="n">
+        <v>10</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>